<commit_message>
added partial draft for my report part
</commit_message>
<xml_diff>
--- a/Reliability Growth Testing/SFRAT Input FD3.xlsx
+++ b/Reliability Growth Testing/SFRAT Input FD3.xlsx
@@ -356,7 +356,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -378,7 +378,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -395,11 +395,11 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
-        <f>A2+1</f>
-        <v>2</v>
+        <f t="shared" ref="A3:A15" si="0">A2+1</f>
+        <v>4</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -413,8 +413,8 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
-        <f t="shared" ref="A4:A17" si="0">A3+1</f>
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="B4">
         <v>2</v>
@@ -432,7 +432,7 @@
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -450,7 +450,7 @@
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6">
         <v>2</v>
@@ -468,10 +468,10 @@
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -486,10 +486,10 @@
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -504,7 +504,7 @@
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B9">
         <v>2</v>
@@ -522,10 +522,10 @@
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -540,10 +540,10 @@
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -558,10 +558,10 @@
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -576,7 +576,7 @@
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -594,10 +594,10 @@
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -612,7 +612,7 @@
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B15">
         <v>1</v>
@@ -624,42 +624,6 @@
         <v>1</v>
       </c>
       <c r="E15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
-      <c r="E17">
         <v>1</v>
       </c>
     </row>

</xml_diff>